<commit_message>
datasheet update & file cleaning & display device pcb design
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="12720"/>
+    <workbookView windowWidth="28540" windowHeight="12720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
     <t>Stepper Motor</t>
   </si>
   <si>
-    <t>5V DC Geared Stepper Motor</t>
+    <t>x27 stepper motor</t>
   </si>
   <si>
     <r>
@@ -101,6 +101,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">ULN2003 Module </t>
     </r>
     <r>
@@ -925,7 +931,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -957,9 +963,6 @@
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
@@ -1541,7 +1544,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="53.75" spans="1:10">
+    <row r="3" ht="36.75" spans="1:10">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -1560,9 +1563,9 @@
       <c r="F3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="12"/>
+      <c r="J3" s="11"/>
     </row>
-    <row r="4" ht="36.75" spans="1:6">
+    <row r="4" ht="18.75" spans="1:6">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -1602,7 +1605,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="36.75" spans="1:6">
+    <row r="6" ht="18.75" spans="1:6">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -1642,7 +1645,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" ht="36.75" spans="1:6">
+    <row r="8" ht="18.75" spans="1:6">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -1662,7 +1665,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" ht="36" spans="1:6">
+    <row r="9" ht="36.75" spans="1:6">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -1702,7 +1705,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" ht="36.75" spans="1:6">
+    <row r="11" ht="18.75" spans="1:6">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -1715,7 +1718,7 @@
       <c r="D11" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="8" t="s">
         <v>41</v>
       </c>
       <c r="F11" s="9" t="s">

</xml_diff>